<commit_message>
Add Georgia music education job-search dashboard
</commit_message>
<xml_diff>
--- a/Career-Research/Technical-Audio-Employer-Master-List/Technical-Audio-Employer-Master-List.xlsx
+++ b/Career-Research/Technical-Audio-Employer-Master-List/Technical-Audio-Employer-Master-List.xlsx
@@ -2,13 +2,57 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7bff1cd69d034352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employer Master" sheetId="2" r:id="Ref31971980644b60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Dashboard" sheetId="3" r:id="R622e668eaf5a4b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Employers" sheetId="4" r:id="R4b6bcaec1c154ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions &amp; Search Guide" sheetId="5" r:id="Ra05f8588da3a48a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R69be011b123d4aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employer Master" sheetId="2" r:id="Rd5075c1139034dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Dashboard" sheetId="3" r:id="R46d0008fcccb43ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consulting Employers" sheetId="4" r:id="Rc888d9be52114849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions &amp; Search Guide" sheetId="5" r:id="Rb699cfb6ed6a4701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Ed Dashboard" sheetId="6" r:id="R07b77a7905d541f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GA District Targets" sheetId="7" r:id="R6832eeeacf8d4900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Music Leads" sheetId="8" r:id="R23ff3c6c4553429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certification Plan" sheetId="9" r:id="R805ac5f042844804"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={E6673A0A-EC28-436B-EA8E-E0580C05AAA7}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="A17" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source supplied by Kevin: GMEA Music Program Leaders Canva resource site.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={A7C26F75-8E4E-2FFA-81E1-40859FDFA8F6}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="A1" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Vacancies are time-sensitive. Recheck the official district portal immediately before applying.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17,7 +61,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="12">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +133,31 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Display"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1D3F66"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D3F66"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0563C1"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,8 +194,28 @@
         <x:fgColor rgb="FF70AD47"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D3F66"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="6">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -155,11 +245,29 @@
         <x:color rgb="FFD9EAD3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="102">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -286,25 +394,115 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF1B5E20"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6E0B4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -315,12 +513,67 @@
         <x:color rgb="FF1B5E20"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6E0B4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF375623"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF375623"/>
+      </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE2F0D9"/>
@@ -329,6 +582,12 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="Kevin Worley" id="{F15ADE75-C747-4DBA-A80C-39FA32BAD3C2}"/>
+</xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -374,6 +633,77 @@
     <x:tableColumn id="14" name="Contact / referral"/>
     <x:tableColumn id="15" name="Next action"/>
     <x:tableColumn id="16" name="Last checked"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MusicEdMetrics" displayName="MusicEdMetrics" ref="A6:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="2">
+    <x:tableColumn id="1" name="Metric"/>
+    <x:tableColumn id="2" name="Count"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="GADistrictTargets" displayName="GADistrictTargets" ref="A1:O24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="Region"/>
+    <x:tableColumn id="2" name="School system"/>
+    <x:tableColumn id="3" name="Hub / area"/>
+    <x:tableColumn id="4" name="Atlanta proximity"/>
+    <x:tableColumn id="5" name="Kevin priority"/>
+    <x:tableColumn id="6" name="Why it fits"/>
+    <x:tableColumn id="7" name="Search terms / route"/>
+    <x:tableColumn id="8" name="Opening signal"/>
+    <x:tableColumn id="9" name="Careers / vacancies URL"/>
+    <x:tableColumn id="10" name="TeachGeorgia music"/>
+    <x:tableColumn id="11" name="GMEA jobs"/>
+    <x:tableColumn id="12" name="Last checked"/>
+    <x:tableColumn id="13" name="Notes"/>
+    <x:tableColumn id="14" name="Application status"/>
+    <x:tableColumn id="15" name="Next review"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CurrentMusicLeads" displayName="CurrentMusicLeads" ref="A1:M11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Priority"/>
+    <x:tableColumn id="2" name="System"/>
+    <x:tableColumn id="3" name="School / site"/>
+    <x:tableColumn id="4" name="Position"/>
+    <x:tableColumn id="5" name="Music area"/>
+    <x:tableColumn id="6" name="Location"/>
+    <x:tableColumn id="7" name="School year"/>
+    <x:tableColumn id="8" name="Status"/>
+    <x:tableColumn id="9" name="Closing date"/>
+    <x:tableColumn id="10" name="Source type"/>
+    <x:tableColumn id="11" name="Posting / search URL"/>
+    <x:tableColumn id="12" name="Last checked"/>
+    <x:tableColumn id="13" name="Verification / fit note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CertificationOptions" displayName="CertificationOptions" ref="A6:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Stage"/>
+    <x:tableColumn id="2" name="Field / action"/>
+    <x:tableColumn id="3" name="Possible route"/>
+    <x:tableColumn id="4" name="Timing"/>
+    <x:tableColumn id="5" name="Career value"/>
+    <x:tableColumn id="6" name="Important limitation"/>
+    <x:tableColumn id="7" name="Authority"/>
+    <x:tableColumn id="8" name="Official URL"/>
+    <x:tableColumn id="9" name="Priority"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -570,6 +900,22 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="A17" dT="2026-08-01T21:34:43.895" personId="{F15ADE75-C747-4DBA-A80C-39FA32BAD3C2}" id="{E6673A0A-EC28-436B-EA8E-E0580C05AAA7}">
+    <xltc:text>Source supplied by Kevin: GMEA Music Program Leaders Canva resource site.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
+<file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="A1" dT="2026-08-01T21:34:43.895" personId="{F15ADE75-C747-4DBA-A80C-39FA32BAD3C2}" id="{A7C26F75-8E4E-2FFA-81E1-40859FDFA8F6}">
+    <xltc:text>Vacancies are time-sensitive. Recheck the official district portal immediately before applying.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -3520,7 +3866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a05764f03e34411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb441eb5fddd4468f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5571,7 +5917,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a7fbd615324645"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda774a3cb6444dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5879,4 +6225,2359 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Georgia Music Education Job Search</x:v>
+      </x:c>
+      <x:c r="B1" s="81"/>
+      <x:c r="C1" s="81"/>
+      <x:c r="D1" s="81"/>
+      <x:c r="E1" s="81"/>
+      <x:c r="F1" s="81"/>
+      <x:c r="G1" s="81"/>
+      <x:c r="H1" s="81"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="81"/>
+      <x:c r="B2" s="81"/>
+      <x:c r="C2" s="81"/>
+      <x:c r="D2" s="81"/>
+      <x:c r="E2" s="81"/>
+      <x:c r="F2" s="81"/>
+      <x:c r="G2" s="81"/>
+      <x:c r="H2" s="81"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="82"/>
+      <x:c r="B3" s="82"/>
+      <x:c r="C3" s="82"/>
+      <x:c r="D3" s="82"/>
+      <x:c r="E3" s="82"/>
+      <x:c r="F3" s="82"/>
+      <x:c r="G3" s="82"/>
+      <x:c r="H3" s="82"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="65" t="str">
+        <x:v>Metro Atlanta priorities, current leads, district portals, and certification planning - updated August 1, 2026</x:v>
+      </x:c>
+      <x:c r="B4" s="65"/>
+      <x:c r="C4" s="65"/>
+      <x:c r="D4" s="65"/>
+      <x:c r="E4" s="65"/>
+      <x:c r="F4" s="65"/>
+      <x:c r="G4" s="65"/>
+      <x:c r="H4" s="65"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="82"/>
+      <x:c r="B5" s="82"/>
+      <x:c r="C5" s="82"/>
+      <x:c r="D5" s="82"/>
+      <x:c r="E5" s="82"/>
+      <x:c r="F5" s="82"/>
+      <x:c r="G5" s="82"/>
+      <x:c r="H5" s="82"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="83" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B6" s="83" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="C6" s="84"/>
+      <x:c r="D6" s="85" t="str">
+        <x:v>Recommended starting sequence</x:v>
+      </x:c>
+      <x:c r="E6" s="85"/>
+      <x:c r="F6" s="85"/>
+      <x:c r="G6" s="85"/>
+      <x:c r="H6" s="85"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="86" t="str">
+        <x:v>District/system targets</x:v>
+      </x:c>
+      <x:c r="B7" s="86" t="n">
+        <x:f>COUNTA('GA District Targets'!B2:B24)</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C7" s="86"/>
+      <x:c r="D7" s="86" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="86" t="str">
+        <x:v>Immediate leads</x:v>
+      </x:c>
+      <x:c r="F7" s="86" t="str">
+        <x:v>Henry assistant band director; Fulton general music; verify APS, DeKalb and Decatur listings.</x:v>
+      </x:c>
+      <x:c r="G7" s="86"/>
+      <x:c r="H7" s="86"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="86" t="str">
+        <x:v>Highest priority</x:v>
+      </x:c>
+      <x:c r="B8" s="86" t="n">
+        <x:f>COUNTIF('GA District Targets'!E2:E24,"Highest")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="86"/>
+      <x:c r="D8" s="86" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E8" s="86" t="str">
+        <x:v>Closest systems</x:v>
+      </x:c>
+      <x:c r="F8" s="86" t="str">
+        <x:v>Cobb and Marietta City; create/refresh profiles and monitor music plus supply/substitute roles.</x:v>
+      </x:c>
+      <x:c r="G8" s="86"/>
+      <x:c r="H8" s="86"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="86" t="str">
+        <x:v>High priority</x:v>
+      </x:c>
+      <x:c r="B9" s="86" t="n">
+        <x:f>COUNTIF('GA District Targets'!E2:E24,"High")</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C9" s="86"/>
+      <x:c r="D9" s="86" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E9" s="86" t="str">
+        <x:v>Large metro systems</x:v>
+      </x:c>
+      <x:c r="F9" s="86" t="str">
+        <x:v>Fulton, APS, DeKalb and Gwinnett; search multiple music-title variants.</x:v>
+      </x:c>
+      <x:c r="G9" s="86"/>
+      <x:c r="H9" s="86"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="86" t="str">
+        <x:v>Current/recent music leads</x:v>
+      </x:c>
+      <x:c r="B10" s="86" t="n">
+        <x:f>COUNTA('Current Music Leads'!B2:B11)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C10" s="86"/>
+      <x:c r="D10" s="86" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E10" s="86" t="str">
+        <x:v>Outer metro</x:v>
+      </x:c>
+      <x:c r="F10" s="86" t="str">
+        <x:v>Cherokee, Paulding, Douglas, Fayette, Henry, Coweta, Rockdale, Forsyth and Buford City.</x:v>
+      </x:c>
+      <x:c r="G10" s="86"/>
+      <x:c r="H10" s="86"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="86" t="str">
+        <x:v>Time-sensitive leads</x:v>
+      </x:c>
+      <x:c r="B11" s="86" t="n">
+        <x:f>COUNTIF('Current Music Leads'!H2:H11,"Closing soon")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" s="86"/>
+      <x:c r="D11" s="86" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E11" s="86" t="str">
+        <x:v>Credential maintenance</x:v>
+      </x:c>
+      <x:c r="F11" s="86" t="str">
+        <x:v>Confirm Music P-12 status/renewal in MyPSC before representing it as active.</x:v>
+      </x:c>
+      <x:c r="G11" s="86"/>
+      <x:c r="H11" s="86"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="86"/>
+      <x:c r="B12" s="86"/>
+      <x:c r="C12" s="86"/>
+      <x:c r="D12" s="86" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E12" s="86" t="str">
+        <x:v>Later additions</x:v>
+      </x:c>
+      <x:c r="F12" s="86" t="str">
+        <x:v>Explore other fields only when a real role and GaPSC pathway justify the effort.</x:v>
+      </x:c>
+      <x:c r="G12" s="86"/>
+      <x:c r="H12" s="86"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="86"/>
+      <x:c r="B13" s="86"/>
+      <x:c r="C13" s="86"/>
+      <x:c r="D13" s="86"/>
+      <x:c r="E13" s="86"/>
+      <x:c r="F13" s="86"/>
+      <x:c r="G13" s="86"/>
+      <x:c r="H13" s="86"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="87" t="str">
+        <x:v>Core search and professional resources</x:v>
+      </x:c>
+      <x:c r="B14" s="87"/>
+      <x:c r="C14" s="87"/>
+      <x:c r="D14" s="87"/>
+      <x:c r="E14" s="87"/>
+      <x:c r="F14" s="87"/>
+      <x:c r="G14" s="87"/>
+      <x:c r="H14" s="87"/>
+    </x:row>
+    <x:row r="15" ht="32" customHeight="1">
+      <x:c r="A15" s="88" t="str">
+        <x:v>TeachGeorgia music search</x:v>
+      </x:c>
+      <x:c r="B15" s="89" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="C15" s="86" t="str">
+        <x:v>Official state database of certified public-school vacancies</x:v>
+      </x:c>
+      <x:c r="D15" s="86"/>
+      <x:c r="E15" s="86"/>
+      <x:c r="F15" s="86"/>
+      <x:c r="G15" s="86"/>
+      <x:c r="H15" s="86"/>
+    </x:row>
+    <x:row r="16" ht="32" customHeight="1">
+      <x:c r="A16" s="88" t="str">
+        <x:v>GMEA Job Listings</x:v>
+      </x:c>
+      <x:c r="B16" s="89" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="C16" s="86" t="str">
+        <x:v>Music-specific statewide job board</x:v>
+      </x:c>
+      <x:c r="D16" s="86"/>
+      <x:c r="E16" s="86"/>
+      <x:c r="F16" s="86"/>
+      <x:c r="G16" s="86"/>
+      <x:c r="H16" s="86"/>
+    </x:row>
+    <x:row r="17" ht="32" customHeight="1">
+      <x:c r="A17" s="88" t="str">
+        <x:v>GMEA Music Program Leaders site</x:v>
+      </x:c>
+      <x:c r="B17" s="89" t="str">
+        <x:v>https://www.canva.com/design/DAG-ZhFBeW8/AyMElDExAaQHD1Vzdx_VnA/edit</x:v>
+      </x:c>
+      <x:c r="C17" s="86" t="str">
+        <x:v>Hiring-process and music-program leadership resources supplied by Kevin</x:v>
+      </x:c>
+      <x:c r="D17" s="86"/>
+      <x:c r="E17" s="86"/>
+      <x:c r="F17" s="86"/>
+      <x:c r="G17" s="86"/>
+      <x:c r="H17" s="86"/>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="88" t="str">
+        <x:v>GMEA Hiring Presentation</x:v>
+      </x:c>
+      <x:c r="B18" s="89" t="str">
+        <x:v>https://www.canva.com/design/DAF6z3_to9A/M5C_uCFrla-K91xIhbkiNA/view?utm_content=DAF6z3_to9A&amp;utm_campaign=designshare&amp;utm_medium=link2&amp;utm_source=uniquelinks&amp;utlId=h2497d648e4</x:v>
+      </x:c>
+      <x:c r="C18" s="86" t="str">
+        <x:v>Resume, interview and hiring-process presentation linked from the Canva site</x:v>
+      </x:c>
+      <x:c r="D18" s="86"/>
+      <x:c r="E18" s="86"/>
+      <x:c r="F18" s="86"/>
+      <x:c r="G18" s="86"/>
+      <x:c r="H18" s="86"/>
+    </x:row>
+    <x:row r="19" ht="32" customHeight="1">
+      <x:c r="A19" s="88" t="str">
+        <x:v>GaDOE Fine Arts Quick Links</x:v>
+      </x:c>
+      <x:c r="B19" s="89" t="str">
+        <x:v>https://linktr.ee/GaDoeFineArts</x:v>
+      </x:c>
+      <x:c r="C19" s="86" t="str">
+        <x:v>State fine-arts resources and supports</x:v>
+      </x:c>
+      <x:c r="D19" s="86"/>
+      <x:c r="E19" s="86"/>
+      <x:c r="F19" s="86"/>
+      <x:c r="G19" s="86"/>
+      <x:c r="H19" s="86"/>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="90" t="str">
+        <x:v>GaPSC / MyPSC</x:v>
+      </x:c>
+      <x:c r="B20" s="91" t="str">
+        <x:v>https://www.gapsc.com/</x:v>
+      </x:c>
+      <x:c r="C20" s="92" t="str">
+        <x:v>Certification, renewal and add-a-field authority</x:v>
+      </x:c>
+      <x:c r="D20" s="92"/>
+      <x:c r="E20" s="92"/>
+      <x:c r="F20" s="92"/>
+      <x:c r="G20" s="92"/>
+      <x:c r="H20" s="92"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A4:H4"/>
+    <x:mergeCell ref="D6:H6"/>
+    <x:mergeCell ref="A14:H14"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18d4c710b897473e"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb44d707ec2694e51"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="44" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="29" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="45" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="94" t="str">
+        <x:v>Region</x:v>
+      </x:c>
+      <x:c r="B1" s="94" t="str">
+        <x:v>School system</x:v>
+      </x:c>
+      <x:c r="C1" s="94" t="str">
+        <x:v>Hub / area</x:v>
+      </x:c>
+      <x:c r="D1" s="94" t="str">
+        <x:v>Atlanta proximity</x:v>
+      </x:c>
+      <x:c r="E1" s="94" t="str">
+        <x:v>Kevin priority</x:v>
+      </x:c>
+      <x:c r="F1" s="94" t="str">
+        <x:v>Why it fits</x:v>
+      </x:c>
+      <x:c r="G1" s="94" t="str">
+        <x:v>Search terms / route</x:v>
+      </x:c>
+      <x:c r="H1" s="94" t="str">
+        <x:v>Opening signal</x:v>
+      </x:c>
+      <x:c r="I1" s="94" t="str">
+        <x:v>Careers / vacancies URL</x:v>
+      </x:c>
+      <x:c r="J1" s="94" t="str">
+        <x:v>TeachGeorgia music</x:v>
+      </x:c>
+      <x:c r="K1" s="94" t="str">
+        <x:v>GMEA jobs</x:v>
+      </x:c>
+      <x:c r="L1" s="94" t="str">
+        <x:v>Last checked</x:v>
+      </x:c>
+      <x:c r="M1" s="94" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="N1" s="94" t="str">
+        <x:v>Application status</x:v>
+      </x:c>
+      <x:c r="O1" s="94" t="str">
+        <x:v>Next review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="52" customHeight="1">
+      <x:c r="A2" s="95" t="str">
+        <x:v>West/Northwest</x:v>
+      </x:c>
+      <x:c r="B2" s="95" t="str">
+        <x:v>Cobb County School District</x:v>
+      </x:c>
+      <x:c r="C2" s="95" t="str">
+        <x:v>Marietta / Cobb</x:v>
+      </x:c>
+      <x:c r="D2" s="95" t="str">
+        <x:v>Core metro; school-dependent</x:v>
+      </x:c>
+      <x:c r="E2" s="95" t="str">
+        <x:v>Highest</x:v>
+      </x:c>
+      <x:c r="F2" s="95" t="str">
+        <x:v>Existing Cobb experience and local network; large music-program footprint</x:v>
+      </x:c>
+      <x:c r="G2" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra, Chorus, General Music and Supply Teacher</x:v>
+      </x:c>
+      <x:c r="H2" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I2" s="97" t="str">
+        <x:v>https://www.cobbk12.org/employment-opportunities</x:v>
+      </x:c>
+      <x:c r="J2" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K2" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L2" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M2" s="95" t="str">
+        <x:v>Best first district from Marietta; also monitor supply and substitute roles.</x:v>
+      </x:c>
+      <x:c r="N2" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O2" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="52" customHeight="1">
+      <x:c r="A3" s="95" t="str">
+        <x:v>West/Northwest</x:v>
+      </x:c>
+      <x:c r="B3" s="95" t="str">
+        <x:v>Marietta City Schools</x:v>
+      </x:c>
+      <x:c r="C3" s="95" t="str">
+        <x:v>Marietta</x:v>
+      </x:c>
+      <x:c r="D3" s="95" t="str">
+        <x:v>Core metro</x:v>
+      </x:c>
+      <x:c r="E3" s="95" t="str">
+        <x:v>Highest</x:v>
+      </x:c>
+      <x:c r="F3" s="95" t="str">
+        <x:v>Closest city system; direct local relevance</x:v>
+      </x:c>
+      <x:c r="G3" s="95" t="str">
+        <x:v>Search Music and Fine Arts; create SchoolSpring profile</x:v>
+      </x:c>
+      <x:c r="H3" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I3" s="97" t="str">
+        <x:v>https://www.marietta-city.org/careers1</x:v>
+      </x:c>
+      <x:c r="J3" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K3" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L3" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M3" s="95" t="str">
+        <x:v>Small system, so openings may be infrequent but highly practical.</x:v>
+      </x:c>
+      <x:c r="N3" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O3" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="52" customHeight="1">
+      <x:c r="A4" s="95" t="str">
+        <x:v>North/Central/South</x:v>
+      </x:c>
+      <x:c r="B4" s="95" t="str">
+        <x:v>Fulton County Schools</x:v>
+      </x:c>
+      <x:c r="C4" s="95" t="str">
+        <x:v>Fulton / Sandy Springs / South Fulton</x:v>
+      </x:c>
+      <x:c r="D4" s="95" t="str">
+        <x:v>Core metro to outer metro</x:v>
+      </x:c>
+      <x:c r="E4" s="95" t="str">
+        <x:v>Highest</x:v>
+      </x:c>
+      <x:c r="F4" s="95" t="str">
+        <x:v>Large system with current general-music lead and broad school geography</x:v>
+      </x:c>
+      <x:c r="G4" s="95" t="str">
+        <x:v>Search Arts-General Music, Band, Orchestra, Chorus and candidate pools</x:v>
+      </x:c>
+      <x:c r="H4" s="95" t="str">
+        <x:v>Current lead visible</x:v>
+      </x:c>
+      <x:c r="I4" s="97" t="str">
+        <x:v>https://jobs.fultonschools.org/go/Teach/8863000/</x:v>
+      </x:c>
+      <x:c r="J4" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K4" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L4" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M4" s="95" t="str">
+        <x:v>Prioritize north/central Fulton locations for commute; evaluate each school separately.</x:v>
+      </x:c>
+      <x:c r="N4" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O4" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="95" t="str">
+        <x:v>Central</x:v>
+      </x:c>
+      <x:c r="B5" s="95" t="str">
+        <x:v>Atlanta Public Schools</x:v>
+      </x:c>
+      <x:c r="C5" s="95" t="str">
+        <x:v>Atlanta</x:v>
+      </x:c>
+      <x:c r="D5" s="95" t="str">
+        <x:v>Core metro</x:v>
+      </x:c>
+      <x:c r="E5" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F5" s="95" t="str">
+        <x:v>Large urban system; music-certified teacher roles and candidate pools</x:v>
+      </x:c>
+      <x:c r="G5" s="95" t="str">
+        <x:v>Search Music Teacher, Band, Orchestra, Chorus and Fine Arts</x:v>
+      </x:c>
+      <x:c r="H5" s="95" t="str">
+        <x:v>Current/recent lead visible</x:v>
+      </x:c>
+      <x:c r="I5" s="97" t="str">
+        <x:v>https://www.applitrack.com/atlantapublicschools/onlineapp/default.aspx?all=1</x:v>
+      </x:c>
+      <x:c r="J5" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K5" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L5" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M5" s="95" t="str">
+        <x:v>Traffic and school location materially change commute.</x:v>
+      </x:c>
+      <x:c r="N5" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O5" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="95" t="str">
+        <x:v>East/Central</x:v>
+      </x:c>
+      <x:c r="B6" s="95" t="str">
+        <x:v>DeKalb County School District</x:v>
+      </x:c>
+      <x:c r="C6" s="95" t="str">
+        <x:v>DeKalb / Decatur / Stone Mountain</x:v>
+      </x:c>
+      <x:c r="D6" s="95" t="str">
+        <x:v>Core metro to outer metro</x:v>
+      </x:c>
+      <x:c r="E6" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F6" s="95" t="str">
+        <x:v>Multiple current/recent elementary music, band and strings leads</x:v>
+      </x:c>
+      <x:c r="G6" s="95" t="str">
+        <x:v>Search Music, Band, Strings, Orchestra, Chorus and split-school roles</x:v>
+      </x:c>
+      <x:c r="H6" s="95" t="str">
+        <x:v>Current/recent leads visible</x:v>
+      </x:c>
+      <x:c r="I6" s="97" t="str">
+        <x:v>https://www.dekalbschoolsga.org/divisions/human-resources/recruitment</x:v>
+      </x:c>
+      <x:c r="J6" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K6" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L6" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M6" s="95" t="str">
+        <x:v>Large, varied district; verify each posting in the district portal.</x:v>
+      </x:c>
+      <x:c r="N6" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O6" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
+      <x:c r="A7" s="95" t="str">
+        <x:v>Central/East</x:v>
+      </x:c>
+      <x:c r="B7" s="95" t="str">
+        <x:v>City Schools of Decatur</x:v>
+      </x:c>
+      <x:c r="C7" s="95" t="str">
+        <x:v>Decatur</x:v>
+      </x:c>
+      <x:c r="D7" s="95" t="str">
+        <x:v>Core metro</x:v>
+      </x:c>
+      <x:c r="E7" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F7" s="95" t="str">
+        <x:v>Current/recent K-2 music lead; compact system</x:v>
+      </x:c>
+      <x:c r="G7" s="95" t="str">
+        <x:v>Search Music and Fine Arts in Frontline</x:v>
+      </x:c>
+      <x:c r="H7" s="95" t="str">
+        <x:v>Current/recent lead visible</x:v>
+      </x:c>
+      <x:c r="I7" s="97" t="str">
+        <x:v>https://www.applitrack.com/csdecatur/onlineapp/default.aspx</x:v>
+      </x:c>
+      <x:c r="J7" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K7" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L7" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M7" s="95" t="str">
+        <x:v>Small district; strong fit when a music opening appears.</x:v>
+      </x:c>
+      <x:c r="N7" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O7" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="95" t="str">
+        <x:v>Northwest</x:v>
+      </x:c>
+      <x:c r="B8" s="95" t="str">
+        <x:v>Cherokee County School District</x:v>
+      </x:c>
+      <x:c r="C8" s="95" t="str">
+        <x:v>Canton / Woodstock</x:v>
+      </x:c>
+      <x:c r="D8" s="95" t="str">
+        <x:v>Approx. 30-60 min; school-dependent</x:v>
+      </x:c>
+      <x:c r="E8" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F8" s="95" t="str">
+        <x:v>Accessible from Marietta; established band/orchestra programs</x:v>
+      </x:c>
+      <x:c r="G8" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra and Chorus; enable job alerts</x:v>
+      </x:c>
+      <x:c r="H8" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I8" s="97" t="str">
+        <x:v>https://www.cherokeek12.net/divisions/human-resources/employment</x:v>
+      </x:c>
+      <x:c r="J8" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K8" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L8" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M8" s="95" t="str">
+        <x:v>Woodstock/south Cherokee generally more practical than far-north schools.</x:v>
+      </x:c>
+      <x:c r="N8" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O8" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="95" t="str">
+        <x:v>West/Northwest</x:v>
+      </x:c>
+      <x:c r="B9" s="95" t="str">
+        <x:v>Paulding County School District</x:v>
+      </x:c>
+      <x:c r="C9" s="95" t="str">
+        <x:v>Dallas / Hiram</x:v>
+      </x:c>
+      <x:c r="D9" s="95" t="str">
+        <x:v>Approx. 30-60 min; school-dependent</x:v>
+      </x:c>
+      <x:c r="E9" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F9" s="95" t="str">
+        <x:v>Practical west-metro commute from Marietta</x:v>
+      </x:c>
+      <x:c r="G9" s="95" t="str">
+        <x:v>Search Music and Fine Arts in SchoolSpring</x:v>
+      </x:c>
+      <x:c r="H9" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I9" s="97" t="str">
+        <x:v>https://paulding.schoolspring.com/</x:v>
+      </x:c>
+      <x:c r="J9" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K9" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L9" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M9" s="95" t="str">
+        <x:v>Consider substitute/supply routes while monitoring certified openings.</x:v>
+      </x:c>
+      <x:c r="N9" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O9" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="95" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="B10" s="95" t="str">
+        <x:v>Douglas County School System</x:v>
+      </x:c>
+      <x:c r="C10" s="95" t="str">
+        <x:v>Douglasville</x:v>
+      </x:c>
+      <x:c r="D10" s="95" t="str">
+        <x:v>Approx. 30-60 min; traffic-dependent</x:v>
+      </x:c>
+      <x:c r="E10" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F10" s="95" t="str">
+        <x:v>Reasonable west-metro target with certified openings portal</x:v>
+      </x:c>
+      <x:c r="G10" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra, Chorus and Elementary Teaching</x:v>
+      </x:c>
+      <x:c r="H10" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I10" s="97" t="str">
+        <x:v>https://www.applitrack.com/douglascounty/onlineapp/default.aspx?all=1</x:v>
+      </x:c>
+      <x:c r="J10" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K10" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L10" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M10" s="95" t="str">
+        <x:v>I-20 traffic can move individual schools outside the intended range.</x:v>
+      </x:c>
+      <x:c r="N10" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O10" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="95" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="B11" s="95" t="str">
+        <x:v>Gwinnett County Public Schools</x:v>
+      </x:c>
+      <x:c r="C11" s="95" t="str">
+        <x:v>Gwinnett / Suwanee</x:v>
+      </x:c>
+      <x:c r="D11" s="95" t="str">
+        <x:v>Approx. 30-60+ min; school-dependent</x:v>
+      </x:c>
+      <x:c r="E11" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F11" s="95" t="str">
+        <x:v>Very large district with broad fine-arts footprint</x:v>
+      </x:c>
+      <x:c r="G11" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra, Chorus and General Music</x:v>
+      </x:c>
+      <x:c r="H11" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I11" s="97" t="str">
+        <x:v>https://www.gcpsk12.org/about-us/careers</x:v>
+      </x:c>
+      <x:c r="J11" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K11" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L11" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M11" s="95" t="str">
+        <x:v>Prioritize west/southwest Gwinnett if commute matters.</x:v>
+      </x:c>
+      <x:c r="N11" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O11" s="96" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="95" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="B12" s="95" t="str">
+        <x:v>Clayton County Public Schools</x:v>
+      </x:c>
+      <x:c r="C12" s="95" t="str">
+        <x:v>Jonesboro / Riverdale</x:v>
+      </x:c>
+      <x:c r="D12" s="95" t="str">
+        <x:v>Approx. 30-60 min; traffic-dependent</x:v>
+      </x:c>
+      <x:c r="E12" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F12" s="95" t="str">
+        <x:v>Large district and regular teacher recruitment</x:v>
+      </x:c>
+      <x:c r="G12" s="95" t="str">
+        <x:v>Search Music, Fine Arts and Teacher Pools</x:v>
+      </x:c>
+      <x:c r="H12" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I12" s="97" t="str">
+        <x:v>https://claytoncounty.schoolspring.com/</x:v>
+      </x:c>
+      <x:c r="J12" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K12" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L12" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M12" s="95" t="str">
+        <x:v>Distance from Marietta may be less practical despite Atlanta proximity.</x:v>
+      </x:c>
+      <x:c r="N12" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O12" s="96" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="A13" s="95" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="B13" s="95" t="str">
+        <x:v>Fayette County Public Schools</x:v>
+      </x:c>
+      <x:c r="C13" s="95" t="str">
+        <x:v>Fayetteville / Peachtree City</x:v>
+      </x:c>
+      <x:c r="D13" s="95" t="str">
+        <x:v>Approx. 35-60+ min</x:v>
+      </x:c>
+      <x:c r="E13" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F13" s="95" t="str">
+        <x:v>Music programs plus proximity to Peachtree City technical-audio ecosystem</x:v>
+      </x:c>
+      <x:c r="G13" s="95" t="str">
+        <x:v>Search Music and Fine Arts in Frontline/YOSS</x:v>
+      </x:c>
+      <x:c r="H13" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I13" s="97" t="str">
+        <x:v>https://www.applitrack.com/fayettega/onlineapp/default.aspx</x:v>
+      </x:c>
+      <x:c r="J13" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K13" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L13" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M13" s="95" t="str">
+        <x:v>Potentially useful geographic overlap with Panasonic/automotive networking.</x:v>
+      </x:c>
+      <x:c r="N13" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O13" s="96" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52" customHeight="1">
+      <x:c r="A14" s="95" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="B14" s="95" t="str">
+        <x:v>Henry County Schools</x:v>
+      </x:c>
+      <x:c r="C14" s="95" t="str">
+        <x:v>McDonough / Stockbridge</x:v>
+      </x:c>
+      <x:c r="D14" s="95" t="str">
+        <x:v>Approx. 35-60+ min; traffic-dependent</x:v>
+      </x:c>
+      <x:c r="E14" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F14" s="95" t="str">
+        <x:v>Current assistant band director lead; large system</x:v>
+      </x:c>
+      <x:c r="G14" s="95" t="str">
+        <x:v>Search Band, Music, Orchestra, Chorus and Fine Arts</x:v>
+      </x:c>
+      <x:c r="H14" s="95" t="str">
+        <x:v>Time-sensitive current lead</x:v>
+      </x:c>
+      <x:c r="I14" s="97" t="str">
+        <x:v>https://www.henry.k12.ga.us/careers</x:v>
+      </x:c>
+      <x:c r="J14" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K14" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L14" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M14" s="95" t="str">
+        <x:v>Assistant Band Director listed on TeachGeorgia with Aug. 3 closing date.</x:v>
+      </x:c>
+      <x:c r="N14" s="95" t="str">
+        <x:v>Review now</x:v>
+      </x:c>
+      <x:c r="O14" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="95" t="str">
+        <x:v>Southwest</x:v>
+      </x:c>
+      <x:c r="B15" s="95" t="str">
+        <x:v>Coweta County School System</x:v>
+      </x:c>
+      <x:c r="C15" s="95" t="str">
+        <x:v>Newnan</x:v>
+      </x:c>
+      <x:c r="D15" s="95" t="str">
+        <x:v>Approx. 40-60+ min</x:v>
+      </x:c>
+      <x:c r="E15" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F15" s="95" t="str">
+        <x:v>Growing system; viable south/west option</x:v>
+      </x:c>
+      <x:c r="G15" s="95" t="str">
+        <x:v>Search Music and Fine Arts in Frontline</x:v>
+      </x:c>
+      <x:c r="H15" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I15" s="97" t="str">
+        <x:v>https://www.applitrack.com/cowetaschools/OnlineApp/default.aspx</x:v>
+      </x:c>
+      <x:c r="J15" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K15" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L15" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M15" s="95" t="str">
+        <x:v>Evaluate school location and I-85 commute individually.</x:v>
+      </x:c>
+      <x:c r="N15" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O15" s="96" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="A16" s="95" t="str">
+        <x:v>East</x:v>
+      </x:c>
+      <x:c r="B16" s="95" t="str">
+        <x:v>Rockdale County Public Schools</x:v>
+      </x:c>
+      <x:c r="C16" s="95" t="str">
+        <x:v>Conyers</x:v>
+      </x:c>
+      <x:c r="D16" s="95" t="str">
+        <x:v>Approx. 35-60+ min</x:v>
+      </x:c>
+      <x:c r="E16" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F16" s="95" t="str">
+        <x:v>Certified vacancy portal and daily postings</x:v>
+      </x:c>
+      <x:c r="G16" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra, Chorus and Certified Vacancies</x:v>
+      </x:c>
+      <x:c r="H16" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I16" s="97" t="str">
+        <x:v>https://www.rockdaleschools.org/departments/human-resources/certified-vacancies</x:v>
+      </x:c>
+      <x:c r="J16" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K16" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L16" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M16" s="95" t="str">
+        <x:v>Outer-east commute may exceed target from Marietta.</x:v>
+      </x:c>
+      <x:c r="N16" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O16" s="96" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="52" customHeight="1">
+      <x:c r="A17" s="95" t="str">
+        <x:v>North</x:v>
+      </x:c>
+      <x:c r="B17" s="95" t="str">
+        <x:v>Forsyth County Schools</x:v>
+      </x:c>
+      <x:c r="C17" s="95" t="str">
+        <x:v>Cumming / Forsyth</x:v>
+      </x:c>
+      <x:c r="D17" s="95" t="str">
+        <x:v>Approx. 35-60+ min</x:v>
+      </x:c>
+      <x:c r="E17" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F17" s="95" t="str">
+        <x:v>Growing north-metro district and strong program potential</x:v>
+      </x:c>
+      <x:c r="G17" s="95" t="str">
+        <x:v>Search Music, Band, Orchestra, Chorus and Certified Educator</x:v>
+      </x:c>
+      <x:c r="H17" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I17" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="J17" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K17" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L17" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M17" s="95" t="str">
+        <x:v>Use TeachGeorgia until a stable direct careers link is confirmed.</x:v>
+      </x:c>
+      <x:c r="N17" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O17" s="96" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="A18" s="95" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="B18" s="95" t="str">
+        <x:v>Buford City Schools</x:v>
+      </x:c>
+      <x:c r="C18" s="95" t="str">
+        <x:v>Buford</x:v>
+      </x:c>
+      <x:c r="D18" s="95" t="str">
+        <x:v>Approx. 35-60+ min</x:v>
+      </x:c>
+      <x:c r="E18" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F18" s="95" t="str">
+        <x:v>Small high-performing city system</x:v>
+      </x:c>
+      <x:c r="G18" s="95" t="str">
+        <x:v>Search Music and Fine Arts through YOSS</x:v>
+      </x:c>
+      <x:c r="H18" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I18" s="97" t="str">
+        <x:v>https://www.bufordcityschools.org/apps/pages/index.jsp?pREC_ID=2684292&amp;type=d&amp;uREC_ID=1617293</x:v>
+      </x:c>
+      <x:c r="J18" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K18" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L18" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M18" s="95" t="str">
+        <x:v>Infrequent openings; keep as a monitored target.</x:v>
+      </x:c>
+      <x:c r="N18" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O18" s="96" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="52" customHeight="1">
+      <x:c r="A19" s="95" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="B19" s="95" t="str">
+        <x:v>Hall County Schools</x:v>
+      </x:c>
+      <x:c r="C19" s="95" t="str">
+        <x:v>Gainesville / Flowery Branch</x:v>
+      </x:c>
+      <x:c r="D19" s="95" t="str">
+        <x:v>Outer ring; often near/over 1 hr</x:v>
+      </x:c>
+      <x:c r="E19" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F19" s="95" t="str">
+        <x:v>Large regional system with certified portal</x:v>
+      </x:c>
+      <x:c r="G19" s="95" t="str">
+        <x:v>Search Music and Fine Arts in certified openings</x:v>
+      </x:c>
+      <x:c r="H19" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I19" s="97" t="str">
+        <x:v>https://www.hallco.org/web/employment-information/</x:v>
+      </x:c>
+      <x:c r="J19" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K19" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L19" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M19" s="95" t="str">
+        <x:v>Flowery Branch may be more practical than Gainesville-area schools.</x:v>
+      </x:c>
+      <x:c r="N19" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O19" s="96" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52" customHeight="1">
+      <x:c r="A20" s="95" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="B20" s="95" t="str">
+        <x:v>Gainesville City School District</x:v>
+      </x:c>
+      <x:c r="C20" s="95" t="str">
+        <x:v>Gainesville</x:v>
+      </x:c>
+      <x:c r="D20" s="95" t="str">
+        <x:v>Outer ring; often over 1 hr</x:v>
+      </x:c>
+      <x:c r="E20" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F20" s="95" t="str">
+        <x:v>TeachGeorgia showed a current Music teacher lead</x:v>
+      </x:c>
+      <x:c r="G20" s="95" t="str">
+        <x:v>Search Music in Frontline and TeachGeorgia</x:v>
+      </x:c>
+      <x:c r="H20" s="95" t="str">
+        <x:v>Current lead visible</x:v>
+      </x:c>
+      <x:c r="I20" s="97" t="str">
+        <x:v>https://www.applitrack.com/gcssk12/onlineapp/</x:v>
+      </x:c>
+      <x:c r="J20" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K20" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L20" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M20" s="95" t="str">
+        <x:v>Current lead needs direct posting verification before applying.</x:v>
+      </x:c>
+      <x:c r="N20" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O20" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="52" customHeight="1">
+      <x:c r="A21" s="95" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="B21" s="95" t="str">
+        <x:v>Butts County School System</x:v>
+      </x:c>
+      <x:c r="C21" s="95" t="str">
+        <x:v>Jackson</x:v>
+      </x:c>
+      <x:c r="D21" s="95" t="str">
+        <x:v>Outer ring; around/over 1 hr</x:v>
+      </x:c>
+      <x:c r="E21" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="F21" s="95" t="str">
+        <x:v>Current/recent elementary music lead</x:v>
+      </x:c>
+      <x:c r="G21" s="95" t="str">
+        <x:v>Search Elementary Music and Music Teacher</x:v>
+      </x:c>
+      <x:c r="H21" s="95" t="str">
+        <x:v>Current/recent lead visible</x:v>
+      </x:c>
+      <x:c r="I21" s="97" t="str">
+        <x:v>https://www.applitrack.com/butts/onlineapp/default.aspx</x:v>
+      </x:c>
+      <x:c r="J21" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K21" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L21" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M21" s="95" t="str">
+        <x:v>Posting 1615 appeared recently; confirm that it remains open.</x:v>
+      </x:c>
+      <x:c r="N21" s="95" t="str">
+        <x:v>Research</x:v>
+      </x:c>
+      <x:c r="O21" s="96" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="52" customHeight="1">
+      <x:c r="A22" s="95" t="str">
+        <x:v>East</x:v>
+      </x:c>
+      <x:c r="B22" s="95" t="str">
+        <x:v>Newton County Schools</x:v>
+      </x:c>
+      <x:c r="C22" s="95" t="str">
+        <x:v>Covington</x:v>
+      </x:c>
+      <x:c r="D22" s="95" t="str">
+        <x:v>Outer ring; often over 1 hr</x:v>
+      </x:c>
+      <x:c r="E22" s="95" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="F22" s="95" t="str">
+        <x:v>Statewide fallback district</x:v>
+      </x:c>
+      <x:c r="G22" s="95" t="str">
+        <x:v>Search Music in TeachGeorgia</x:v>
+      </x:c>
+      <x:c r="H22" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I22" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="J22" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K22" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L22" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M22" s="95" t="str">
+        <x:v>Keep below closer metro systems unless role is unusually strong.</x:v>
+      </x:c>
+      <x:c r="N22" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O22" s="96" t="n">
+        <x:v>46242</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="52" customHeight="1">
+      <x:c r="A23" s="95" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="B23" s="95" t="str">
+        <x:v>Carrollton City / Carroll County</x:v>
+      </x:c>
+      <x:c r="C23" s="95" t="str">
+        <x:v>Carrollton</x:v>
+      </x:c>
+      <x:c r="D23" s="95" t="str">
+        <x:v>Outer ring; often over 1 hr</x:v>
+      </x:c>
+      <x:c r="E23" s="95" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="F23" s="95" t="str">
+        <x:v>Statewide fallback with established music programs</x:v>
+      </x:c>
+      <x:c r="G23" s="95" t="str">
+        <x:v>Search Music, Band and Fine Arts in TeachGeorgia</x:v>
+      </x:c>
+      <x:c r="H23" s="95" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="I23" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="J23" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K23" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L23" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M23" s="95" t="str">
+        <x:v>Consider only for a particularly strong role or relocation case.</x:v>
+      </x:c>
+      <x:c r="N23" s="95" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="O23" s="96" t="n">
+        <x:v>46242</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="52" customHeight="1">
+      <x:c r="A24" s="95" t="str">
+        <x:v>Southwest</x:v>
+      </x:c>
+      <x:c r="B24" s="95" t="str">
+        <x:v>Troup County School System</x:v>
+      </x:c>
+      <x:c r="C24" s="95" t="str">
+        <x:v>LaGrange</x:v>
+      </x:c>
+      <x:c r="D24" s="95" t="str">
+        <x:v>Beyond 1 hr</x:v>
+      </x:c>
+      <x:c r="E24" s="95" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="F24" s="95" t="str">
+        <x:v>Current Music Teacher lead with Aug. 11 closing date</x:v>
+      </x:c>
+      <x:c r="G24" s="95" t="str">
+        <x:v>Search Music in TeachGeorgia</x:v>
+      </x:c>
+      <x:c r="H24" s="95" t="str">
+        <x:v>Time-sensitive statewide lead</x:v>
+      </x:c>
+      <x:c r="I24" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=All&amp;Systems=7411</x:v>
+      </x:c>
+      <x:c r="J24" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="K24" s="97" t="str">
+        <x:v>https://www.gmea.org/jobs</x:v>
+      </x:c>
+      <x:c r="L24" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M24" s="95" t="str">
+        <x:v>Outside preferred radius; retained as statewide fallback.</x:v>
+      </x:c>
+      <x:c r="N24" s="95" t="str">
+        <x:v>Review if flexible</x:v>
+      </x:c>
+      <x:c r="O24" s="96" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="E2:E24">
+    <x:cfRule type="expression" dxfId="4" priority="1">
+      <x:formula>E2="Highest"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="5" priority="2">
+      <x:formula>E2="High"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E2:E24">
+      <x:formula1>"Highest,High,Medium,Low"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N2:N24">
+      <x:formula1>"Not started,Research,Review now,Review if flexible,Profile created,Applied,Closed"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a3b19716aae4514"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="27" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="46" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="49" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="93" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="B1" s="93" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="C1" s="93" t="str">
+        <x:v>School / site</x:v>
+      </x:c>
+      <x:c r="D1" s="93" t="str">
+        <x:v>Position</x:v>
+      </x:c>
+      <x:c r="E1" s="93" t="str">
+        <x:v>Music area</x:v>
+      </x:c>
+      <x:c r="F1" s="93" t="str">
+        <x:v>Location</x:v>
+      </x:c>
+      <x:c r="G1" s="93" t="str">
+        <x:v>School year</x:v>
+      </x:c>
+      <x:c r="H1" s="93" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="I1" s="93" t="str">
+        <x:v>Closing date</x:v>
+      </x:c>
+      <x:c r="J1" s="93" t="str">
+        <x:v>Source type</x:v>
+      </x:c>
+      <x:c r="K1" s="93" t="str">
+        <x:v>Posting / search URL</x:v>
+      </x:c>
+      <x:c r="L1" s="93" t="str">
+        <x:v>Last checked</x:v>
+      </x:c>
+      <x:c r="M1" s="93" t="str">
+        <x:v>Verification / fit note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="95" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="B2" s="95" t="str">
+        <x:v>Fulton County Schools</x:v>
+      </x:c>
+      <x:c r="C2" s="95" t="str">
+        <x:v>High Point Elementary</x:v>
+      </x:c>
+      <x:c r="D2" s="95" t="str">
+        <x:v>Teacher, Arts-General Music</x:v>
+      </x:c>
+      <x:c r="E2" s="95" t="str">
+        <x:v>General Music</x:v>
+      </x:c>
+      <x:c r="F2" s="95" t="str">
+        <x:v>Atlanta / Fulton</x:v>
+      </x:c>
+      <x:c r="G2" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H2" s="95" t="str">
+        <x:v>Open/verify</x:v>
+      </x:c>
+      <x:c r="I2" s="96" t="str">
+        <x:v>Not shown</x:v>
+      </x:c>
+      <x:c r="J2" s="95" t="str">
+        <x:v>Official Fulton careers</x:v>
+      </x:c>
+      <x:c r="K2" s="97" t="str">
+        <x:v>https://jobs.fultonschools.org/go/View-All-Jobs/8863400/</x:v>
+      </x:c>
+      <x:c r="L2" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M2" s="95" t="str">
+        <x:v>Posting ID 35018 visible in official search; inspect exact school/location before applying.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="54" customHeight="1">
+      <x:c r="A3" s="95" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="B3" s="95" t="str">
+        <x:v>Henry County Schools</x:v>
+      </x:c>
+      <x:c r="C3" s="95" t="str">
+        <x:v>School not shown in index</x:v>
+      </x:c>
+      <x:c r="D3" s="95" t="str">
+        <x:v>Assistant Band Director</x:v>
+      </x:c>
+      <x:c r="E3" s="95" t="str">
+        <x:v>Band</x:v>
+      </x:c>
+      <x:c r="F3" s="95" t="str">
+        <x:v>Henry County</x:v>
+      </x:c>
+      <x:c r="G3" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H3" s="95" t="str">
+        <x:v>Closing soon</x:v>
+      </x:c>
+      <x:c r="I3" s="96" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="J3" s="95" t="str">
+        <x:v>TeachGeorgia official state database</x:v>
+      </x:c>
+      <x:c r="K3" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=100&amp;Systems=All</x:v>
+      </x:c>
+      <x:c r="L3" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M3" s="95" t="str">
+        <x:v>Time-sensitive; open the state listing immediately and verify requirements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B4" s="95" t="str">
+        <x:v>Atlanta Public Schools</x:v>
+      </x:c>
+      <x:c r="C4" s="95" t="str">
+        <x:v>District posting</x:v>
+      </x:c>
+      <x:c r="D4" s="95" t="str">
+        <x:v>Music Teacher</x:v>
+      </x:c>
+      <x:c r="E4" s="95" t="str">
+        <x:v>Music P-12</x:v>
+      </x:c>
+      <x:c r="F4" s="95" t="str">
+        <x:v>Atlanta</x:v>
+      </x:c>
+      <x:c r="G4" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H4" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I4" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J4" s="95" t="str">
+        <x:v>Official APS Frontline</x:v>
+      </x:c>
+      <x:c r="K4" s="97" t="str">
+        <x:v>https://www.applitrack.com/atlantapublicschools/onlineapp/default.aspx?all=1</x:v>
+      </x:c>
+      <x:c r="L4" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M4" s="95" t="str">
+        <x:v>Portal text indicates GA Music Teacher certification K-12; locate exact JobID and school.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B5" s="95" t="str">
+        <x:v>DeKalb County School District</x:v>
+      </x:c>
+      <x:c r="C5" s="95" t="str">
+        <x:v>Chesnut Elementary</x:v>
+      </x:c>
+      <x:c r="D5" s="95" t="str">
+        <x:v>Band/Strings Teacher</x:v>
+      </x:c>
+      <x:c r="E5" s="95" t="str">
+        <x:v>Band and Strings</x:v>
+      </x:c>
+      <x:c r="F5" s="95" t="str">
+        <x:v>DeKalb</x:v>
+      </x:c>
+      <x:c r="G5" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H5" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I5" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J5" s="95" t="str">
+        <x:v>District/aggregated listing</x:v>
+      </x:c>
+      <x:c r="K5" s="97" t="str">
+        <x:v>https://www.dekalbschoolsga.org/divisions/human-resources/recruitment</x:v>
+      </x:c>
+      <x:c r="L5" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M5" s="95" t="str">
+        <x:v>Verify current status and split-school expectations in DCSD portal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B6" s="95" t="str">
+        <x:v>DeKalb County School District</x:v>
+      </x:c>
+      <x:c r="C6" s="95" t="str">
+        <x:v>Barack Obama Magnet of Technology ES</x:v>
+      </x:c>
+      <x:c r="D6" s="95" t="str">
+        <x:v>Teacher, Music</x:v>
+      </x:c>
+      <x:c r="E6" s="95" t="str">
+        <x:v>Elementary Music</x:v>
+      </x:c>
+      <x:c r="F6" s="95" t="str">
+        <x:v>Atlanta / DeKalb</x:v>
+      </x:c>
+      <x:c r="G6" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H6" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I6" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J6" s="95" t="str">
+        <x:v>District/aggregated listing</x:v>
+      </x:c>
+      <x:c r="K6" s="97" t="str">
+        <x:v>https://www.dekalbschoolsga.org/divisions/human-resources/recruitment</x:v>
+      </x:c>
+      <x:c r="L6" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M6" s="95" t="str">
+        <x:v>Recently indexed as Area 3 elementary music.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B7" s="95" t="str">
+        <x:v>DeKalb County School District</x:v>
+      </x:c>
+      <x:c r="C7" s="95" t="str">
+        <x:v>Smoke Rise Elementary / split locations</x:v>
+      </x:c>
+      <x:c r="D7" s="95" t="str">
+        <x:v>Teacher, Music (Band)</x:v>
+      </x:c>
+      <x:c r="E7" s="95" t="str">
+        <x:v>Elementary Band</x:v>
+      </x:c>
+      <x:c r="F7" s="95" t="str">
+        <x:v>Stone Mountain</x:v>
+      </x:c>
+      <x:c r="G7" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H7" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I7" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J7" s="95" t="str">
+        <x:v>District/aggregated listing</x:v>
+      </x:c>
+      <x:c r="K7" s="97" t="str">
+        <x:v>https://www.dekalbschoolsga.org/divisions/human-resources/recruitment</x:v>
+      </x:c>
+      <x:c r="L7" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M7" s="95" t="str">
+        <x:v>Listing indicated service across four locations; assess travel and schedule carefully.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B8" s="95" t="str">
+        <x:v>City Schools of Decatur</x:v>
+      </x:c>
+      <x:c r="C8" s="95" t="str">
+        <x:v>Oakhurst Elementary</x:v>
+      </x:c>
+      <x:c r="D8" s="95" t="str">
+        <x:v>K-2 Music Teacher</x:v>
+      </x:c>
+      <x:c r="E8" s="95" t="str">
+        <x:v>Elementary General Music</x:v>
+      </x:c>
+      <x:c r="F8" s="95" t="str">
+        <x:v>Decatur</x:v>
+      </x:c>
+      <x:c r="G8" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H8" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I8" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J8" s="95" t="str">
+        <x:v>Official district Frontline</x:v>
+      </x:c>
+      <x:c r="K8" s="97" t="str">
+        <x:v>https://www.applitrack.com/csdecatur/onlineapp/default.aspx</x:v>
+      </x:c>
+      <x:c r="L8" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M8" s="95" t="str">
+        <x:v>Recent indexed listing; confirm open status in Frontline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="B9" s="95" t="str">
+        <x:v>Butts County School System</x:v>
+      </x:c>
+      <x:c r="C9" s="95" t="str">
+        <x:v>Elementary school TBD</x:v>
+      </x:c>
+      <x:c r="D9" s="95" t="str">
+        <x:v>Music Teacher (Elementary)</x:v>
+      </x:c>
+      <x:c r="E9" s="95" t="str">
+        <x:v>Elementary Music</x:v>
+      </x:c>
+      <x:c r="F9" s="95" t="str">
+        <x:v>Jackson</x:v>
+      </x:c>
+      <x:c r="G9" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H9" s="95" t="str">
+        <x:v>Visible current/recent lead</x:v>
+      </x:c>
+      <x:c r="I9" s="96" t="str">
+        <x:v>Until filled/verify</x:v>
+      </x:c>
+      <x:c r="J9" s="95" t="str">
+        <x:v>Official Frontline posting</x:v>
+      </x:c>
+      <x:c r="K9" s="97" t="str">
+        <x:v>https://www.applitrack.com/butts/onlineapp/default.aspx?AppliTrackJobId=1615&amp;AppliTrackLayoutMode=detail&amp;AppliTrackViewPosting=1</x:v>
+      </x:c>
+      <x:c r="L9" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M9" s="95" t="str">
+        <x:v>About 45 miles south of Atlanta; likely outside preferred Marietta commute.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="B10" s="95" t="str">
+        <x:v>Gainesville City School District</x:v>
+      </x:c>
+      <x:c r="C10" s="95" t="str">
+        <x:v>School not shown in index</x:v>
+      </x:c>
+      <x:c r="D10" s="95" t="str">
+        <x:v>Teacher - Music</x:v>
+      </x:c>
+      <x:c r="E10" s="95" t="str">
+        <x:v>Music</x:v>
+      </x:c>
+      <x:c r="F10" s="95" t="str">
+        <x:v>Gainesville</x:v>
+      </x:c>
+      <x:c r="G10" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H10" s="95" t="str">
+        <x:v>Visible in TeachGeorgia</x:v>
+      </x:c>
+      <x:c r="I10" s="96" t="str">
+        <x:v>Verify in portal</x:v>
+      </x:c>
+      <x:c r="J10" s="95" t="str">
+        <x:v>TeachGeorgia + official Frontline</x:v>
+      </x:c>
+      <x:c r="K10" s="97" t="str">
+        <x:v>https://www.applitrack.com/gcssk12/onlineapp/</x:v>
+      </x:c>
+      <x:c r="L10" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M10" s="95" t="str">
+        <x:v>Outside core radius; verify the posting and school before considering.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="95" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="B11" s="95" t="str">
+        <x:v>Troup County School System</x:v>
+      </x:c>
+      <x:c r="C11" s="95" t="str">
+        <x:v>School not shown in index</x:v>
+      </x:c>
+      <x:c r="D11" s="95" t="str">
+        <x:v>Music Teacher</x:v>
+      </x:c>
+      <x:c r="E11" s="95" t="str">
+        <x:v>Music</x:v>
+      </x:c>
+      <x:c r="F11" s="95" t="str">
+        <x:v>LaGrange</x:v>
+      </x:c>
+      <x:c r="G11" s="95" t="str">
+        <x:v>2026-2027</x:v>
+      </x:c>
+      <x:c r="H11" s="95" t="str">
+        <x:v>Closing soon</x:v>
+      </x:c>
+      <x:c r="I11" s="96" t="n">
+        <x:v>46245</x:v>
+      </x:c>
+      <x:c r="J11" s="95" t="str">
+        <x:v>TeachGeorgia official state database</x:v>
+      </x:c>
+      <x:c r="K11" s="97" t="str">
+        <x:v>https://www.teachgeorgia.org/AdvSearch.aspx?Subjects=All&amp;Systems=7411</x:v>
+      </x:c>
+      <x:c r="L11" s="96" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="M11" s="95" t="str">
+        <x:v>Statewide fallback beyond preferred one-hour Atlanta radius.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="H2:H11">
+    <x:cfRule type="expression" dxfId="6" priority="1">
+      <x:formula>H2="Closing soon"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="A2:A11">
+    <x:cfRule type="expression" dxfId="7" priority="2">
+      <x:formula>A2="Immediate"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re99b5a3e75b34002"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f35450bc3243d3"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="53" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="46" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="61" t="str">
+        <x:v>Georgia Certification Strategy</x:v>
+      </x:c>
+      <x:c r="B1" s="61"/>
+      <x:c r="C1" s="61"/>
+      <x:c r="D1" s="61"/>
+      <x:c r="E1" s="61"/>
+      <x:c r="F1" s="61"/>
+      <x:c r="G1" s="61"/>
+      <x:c r="H1" s="61"/>
+      <x:c r="I1" s="61"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="61"/>
+      <x:c r="B2" s="61"/>
+      <x:c r="C2" s="61"/>
+      <x:c r="D2" s="61"/>
+      <x:c r="E2" s="61"/>
+      <x:c r="F2" s="61"/>
+      <x:c r="G2" s="61"/>
+      <x:c r="H2" s="61"/>
+      <x:c r="I2" s="61"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="65" t="str">
+        <x:v>Music P-12 first; other fields only after a real role, individual GaPSC review, and a credible preparation plan</x:v>
+      </x:c>
+      <x:c r="B4" s="65"/>
+      <x:c r="C4" s="65"/>
+      <x:c r="D4" s="65"/>
+      <x:c r="E4" s="65"/>
+      <x:c r="F4" s="65"/>
+      <x:c r="G4" s="65"/>
+      <x:c r="H4" s="65"/>
+      <x:c r="I4" s="65"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="93" t="str">
+        <x:v>Stage</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>Field / action</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Possible route</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>Timing</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>Career value</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Important limitation</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>Authority</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>Official URL</x:v>
+      </x:c>
+      <x:c r="I6" s="93" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="58" customHeight="1">
+      <x:c r="A7" s="95" t="str">
+        <x:v>Current foundation</x:v>
+      </x:c>
+      <x:c r="B7" s="95" t="str">
+        <x:v>Music P-12</x:v>
+      </x:c>
+      <x:c r="C7" s="95" t="str">
+        <x:v>Renew/reactivate as appropriate</x:v>
+      </x:c>
+      <x:c r="D7" s="95" t="str">
+        <x:v>Immediate when employment or application requires it</x:v>
+      </x:c>
+      <x:c r="E7" s="95" t="str">
+        <x:v>Direct match to band, orchestra, chorus and general-music roles</x:v>
+      </x:c>
+      <x:c r="F7" s="95" t="str">
+        <x:v>Confirm current certificate status and renewal path in MyPSC; do not assume an expired certificate renews automatically.</x:v>
+      </x:c>
+      <x:c r="G7" s="95" t="str">
+        <x:v>MyPSC + GaPSC</x:v>
+      </x:c>
+      <x:c r="H7" s="97" t="str">
+        <x:v>https://mypsc.gapsc.org/</x:v>
+      </x:c>
+      <x:c r="I7" s="95" t="str">
+        <x:v>Priority 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="95" t="str">
+        <x:v>Credential maintenance</x:v>
+      </x:c>
+      <x:c r="B8" s="95" t="str">
+        <x:v>Georgia certificate renewal</x:v>
+      </x:c>
+      <x:c r="C8" s="95" t="str">
+        <x:v>Complete current GaPSC renewal requirements</x:v>
+      </x:c>
+      <x:c r="D8" s="95" t="str">
+        <x:v>Immediate</x:v>
+      </x:c>
+      <x:c r="E8" s="95" t="str">
+        <x:v>Keeps existing music field usable</x:v>
+      </x:c>
+      <x:c r="F8" s="95" t="str">
+        <x:v>Use individual MyPSC correspondence and employing-district guidance; requirements depend on certificate/status.</x:v>
+      </x:c>
+      <x:c r="G8" s="95" t="str">
+        <x:v>GaPSC</x:v>
+      </x:c>
+      <x:c r="H8" s="97" t="str">
+        <x:v>https://www.gapsc.com/</x:v>
+      </x:c>
+      <x:c r="I8" s="95" t="str">
+        <x:v>Priority 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="95" t="str">
+        <x:v>Potential add-on</x:v>
+      </x:c>
+      <x:c r="B9" s="95" t="str">
+        <x:v>Computer Science</x:v>
+      </x:c>
+      <x:c r="C9" s="95" t="str">
+        <x:v>Investigate add-a-field route</x:v>
+      </x:c>
+      <x:c r="D9" s="95" t="str">
+        <x:v>Later, if it supports a realistic teaching role</x:v>
+      </x:c>
+      <x:c r="E9" s="95" t="str">
+        <x:v>Connects coding/DSP learning with school technology pathways</x:v>
+      </x:c>
+      <x:c r="F9" s="95" t="str">
+        <x:v>Verify the exact field, grade band and testing/program route in Upgrade Advisor.</x:v>
+      </x:c>
+      <x:c r="G9" s="95" t="str">
+        <x:v>GaPSC Upgrade Advisor</x:v>
+      </x:c>
+      <x:c r="H9" s="97" t="str">
+        <x:v>https://www.gapsc.com/commission/policies_guidelines/UpgradeUtility/Upgrade_Initial.aspx</x:v>
+      </x:c>
+      <x:c r="I9" s="95" t="str">
+        <x:v>Explore</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="95" t="str">
+        <x:v>Potential add-on</x:v>
+      </x:c>
+      <x:c r="B10" s="95" t="str">
+        <x:v>CTAE Audio/Video Technology &amp; Film</x:v>
+      </x:c>
+      <x:c r="C10" s="95" t="str">
+        <x:v>Investigate eligibility and experience requirements</x:v>
+      </x:c>
+      <x:c r="D10" s="95" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="E10" s="95" t="str">
+        <x:v>Closest school subject to technical audio, production and media background</x:v>
+      </x:c>
+      <x:c r="F10" s="95" t="str">
+        <x:v>CTAE fields can have distinct occupational-experience requirements; request an individual GaPSC determination.</x:v>
+      </x:c>
+      <x:c r="G10" s="95" t="str">
+        <x:v>GaPSC</x:v>
+      </x:c>
+      <x:c r="H10" s="97" t="str">
+        <x:v>https://www.gapsc.com/</x:v>
+      </x:c>
+      <x:c r="I10" s="95" t="str">
+        <x:v>Explore carefully</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="95" t="str">
+        <x:v>Potential endorsement</x:v>
+      </x:c>
+      <x:c r="B11" s="95" t="str">
+        <x:v>ESOL</x:v>
+      </x:c>
+      <x:c r="C11" s="95" t="str">
+        <x:v>Investigate approved endorsement/program</x:v>
+      </x:c>
+      <x:c r="D11" s="95" t="str">
+        <x:v>Later if district demand and workload justify it</x:v>
+      </x:c>
+      <x:c r="E11" s="95" t="str">
+        <x:v>Useful across diverse metro districts and may broaden assignment flexibility</x:v>
+      </x:c>
+      <x:c r="F11" s="95" t="str">
+        <x:v>An endorsement is not interchangeable with every stand-alone teaching field; verify program requirements.</x:v>
+      </x:c>
+      <x:c r="G11" s="95" t="str">
+        <x:v>GaPSC Add-a-Field Rule</x:v>
+      </x:c>
+      <x:c r="H11" s="97" t="str">
+        <x:v>https://www.gapsc.com/Rules/Current/Certification/505-2-.34.pdf</x:v>
+      </x:c>
+      <x:c r="I11" s="95" t="str">
+        <x:v>Optional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="95" t="str">
+        <x:v>Potential add-on</x:v>
+      </x:c>
+      <x:c r="B12" s="95" t="str">
+        <x:v>Special Education</x:v>
+      </x:c>
+      <x:c r="C12" s="95" t="str">
+        <x:v>Consider only with genuine interest and preparation</x:v>
+      </x:c>
+      <x:c r="D12" s="95" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="E12" s="95" t="str">
+        <x:v>High-demand field and may complement inclusive music teaching</x:v>
+      </x:c>
+      <x:c r="F12" s="95" t="str">
+        <x:v>Substantial responsibility and training; do not pursue solely to increase job volume.</x:v>
+      </x:c>
+      <x:c r="G12" s="95" t="str">
+        <x:v>GaPSC Add-a-Field Rule</x:v>
+      </x:c>
+      <x:c r="H12" s="97" t="str">
+        <x:v>https://www.gapsc.com/Rules/Current/Certification/505-2-.34.pdf</x:v>
+      </x:c>
+      <x:c r="I12" s="95" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="95" t="str">
+        <x:v>Potential add-on</x:v>
+      </x:c>
+      <x:c r="B13" s="95" t="str">
+        <x:v>Mathematics 6-12</x:v>
+      </x:c>
+      <x:c r="C13" s="95" t="str">
+        <x:v>Consider only if content readiness is strong</x:v>
+      </x:c>
+      <x:c r="D13" s="95" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="E13" s="95" t="str">
+        <x:v>Could widen certified openings and connect to technical study</x:v>
+      </x:c>
+      <x:c r="F13" s="95" t="str">
+        <x:v>Passing a test is not the same as classroom readiness; verify pathway and content depth.</x:v>
+      </x:c>
+      <x:c r="G13" s="95" t="str">
+        <x:v>GaPSC Upgrade Advisor</x:v>
+      </x:c>
+      <x:c r="H13" s="97" t="str">
+        <x:v>https://www.gapsc.com/commission/policies_guidelines/UpgradeUtility/Upgrade_Initial.aspx</x:v>
+      </x:c>
+      <x:c r="I13" s="95" t="str">
+        <x:v>Conditional</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
+      <x:c r="A14" s="95" t="str">
+        <x:v>Potential add-on</x:v>
+      </x:c>
+      <x:c r="B14" s="95" t="str">
+        <x:v>Elementary Education P-5</x:v>
+      </x:c>
+      <x:c r="C14" s="95" t="str">
+        <x:v>Program-based investigation</x:v>
+      </x:c>
+      <x:c r="D14" s="95" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="E14" s="95" t="str">
+        <x:v>Would broaden elementary classroom options</x:v>
+      </x:c>
+      <x:c r="F14" s="95" t="str">
+        <x:v>Often requires an approved educator-preparation route rather than a simple test-only addition; verify individually.</x:v>
+      </x:c>
+      <x:c r="G14" s="95" t="str">
+        <x:v>GaPSC Add-a-Field Rule</x:v>
+      </x:c>
+      <x:c r="H14" s="97" t="str">
+        <x:v>https://www.gapsc.com/Rules/Current/Certification/505-2-.34.pdf</x:v>
+      </x:c>
+      <x:c r="I14" s="95" t="str">
+        <x:v>Low priority</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="101" t="str">
+        <x:v>Planning rule: Do not invest in another certification field merely to increase the number of possible applications. Confirm the role demand, the GaPSC pathway, the preparation burden, and whether you would genuinely accept and sustain that teaching assignment.</x:v>
+      </x:c>
+      <x:c r="B16" s="101"/>
+      <x:c r="C16" s="101"/>
+      <x:c r="D16" s="101"/>
+      <x:c r="E16" s="101"/>
+      <x:c r="F16" s="101"/>
+      <x:c r="G16" s="101"/>
+      <x:c r="H16" s="101"/>
+      <x:c r="I16" s="101"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="101"/>
+      <x:c r="B17" s="101"/>
+      <x:c r="C17" s="101"/>
+      <x:c r="D17" s="101"/>
+      <x:c r="E17" s="101"/>
+      <x:c r="F17" s="101"/>
+      <x:c r="G17" s="101"/>
+      <x:c r="H17" s="101"/>
+      <x:c r="I17" s="101"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I2"/>
+    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="A16:I17"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="I7:I14">
+    <x:cfRule type="expression" dxfId="8" priority="1">
+      <x:formula>I7="Priority 1"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201bc89f891041a0"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>